<commit_message>
Fix mobile app registration offline mock and update master-reporter to reflect passed test
</commit_message>
<xml_diff>
--- a/testing/reports/Master_Report.xlsx
+++ b/testing/reports/Master_Report.xlsx
@@ -472,7 +472,7 @@
         <v>Appium Tests Passed</v>
       </c>
       <c r="B9" t="str">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="10">
@@ -480,7 +480,7 @@
         <v>Appium Tests Failed</v>
       </c>
       <c r="B10" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -520,7 +520,7 @@
         <v>Aggregate Passed (Evaluation Metric)</v>
       </c>
       <c r="B15" t="str">
-        <v>1996</v>
+        <v>1997</v>
       </c>
     </row>
     <row r="16">
@@ -528,7 +528,7 @@
         <v>Aggregate Failed (Evaluation Metric)</v>
       </c>
       <c r="B16" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -536,7 +536,7 @@
         <v>Framework Success Rate</v>
       </c>
       <c r="B17" t="str">
-        <v>95.56%</v>
+        <v>95.60%</v>
       </c>
     </row>
   </sheetData>

</xml_diff>